<commit_message>
fix(release): harden auth and private media flows
</commit_message>
<xml_diff>
--- a/public/template-acoes-pontuais.xlsx
+++ b/public/template-acoes-pontuais.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
   <si>
     <t>Evento *</t>
   </si>
@@ -38,24 +38,6 @@
     <t>Resultados *</t>
   </si>
   <si>
-    <t>Foto 1 - URL Dropbox</t>
-  </si>
-  <si>
-    <t>Foto 1 - Legenda</t>
-  </si>
-  <si>
-    <t>Foto 2 - URL Dropbox</t>
-  </si>
-  <si>
-    <t>Foto 2 - Legenda</t>
-  </si>
-  <si>
-    <t>Foto 3 - URL Dropbox</t>
-  </si>
-  <si>
-    <t>Foto 3 - Legenda</t>
-  </si>
-  <si>
     <t>Monitoramento emergencial - Floração de cianobactérias</t>
   </si>
   <si>
@@ -80,39 +62,21 @@
     <t>Clorofila-a 38,2 µg/L; presença de Microcystis aeruginosa.</t>
   </si>
   <si>
-    <t>https://dropbox.com/s/exemplo1</t>
-  </si>
-  <si>
-    <t>Vista geral da floração na margem leste</t>
-  </si>
-  <si>
-    <t>https://dropbox.com/s/exemplo2</t>
-  </si>
-  <si>
-    <t>Coleta superficial - ponto P1</t>
+    <t>-25.4310</t>
+  </si>
+  <si>
+    <t>-49.6755</t>
+  </si>
+  <si>
+    <t>Clorofila-a 12,4 µg/L; ausência de organismos visíveis.</t>
+  </si>
+  <si>
+    <t>INSTRUÇÕES DE PREENCHIMENTO - Ações Pontuais (Yva'e Monitoramento)</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>-25.4310</t>
-  </si>
-  <si>
-    <t>-49.6755</t>
-  </si>
-  <si>
-    <t>Clorofila-a 12,4 µg/L; ausência de organismos visíveis.</t>
-  </si>
-  <si>
-    <t>https://dropbox.com/s/exemplo3</t>
-  </si>
-  <si>
-    <t>Ponto P2 - margem oeste</t>
-  </si>
-  <si>
-    <t>INSTRUÇÕES DE PREENCHIMENTO - Ações Pontuais (Yva'e Monitoramento)</t>
-  </si>
-  <si>
     <t>ESTRUTURA</t>
   </si>
   <si>
@@ -152,16 +116,13 @@
     <t xml:space="preserve">  • Resultados — texto livre com os resultados ou observações da coleta</t>
   </si>
   <si>
-    <t>FOTOS (opcionais)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • É possível anexar até 3 fotos por ponto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • Para cada foto, preencha URL (link Dropbox público) e Legenda.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • Para mais de 3 fotos por ponto, adicione fotos extras pelo formulário do app após a importação.</t>
+    <t>FOTOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Fotos são associadas pelo aplicativo e armazenadas exclusivamente no Supabase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Não inclua links de serviços externos nesta planilha.</t>
   </si>
   <si>
     <t>DICAS</t>
@@ -614,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N503"/>
+  <dimension ref="A1:H503"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -623,15 +584,9 @@
     <col min="4" max="5" width="22" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="36" customWidth="1"/>
-    <col min="10" max="10" width="32" customWidth="1"/>
-    <col min="11" max="11" width="36" customWidth="1"/>
-    <col min="12" max="12" width="32" customWidth="1"/>
-    <col min="13" max="13" width="36" customWidth="1"/>
-    <col min="14" max="14" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="38" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" ht="38" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -656,111 +611,57 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1271,7 +1172,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1279,137 +1180,132 @@
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>26</v>
+      <c r="A22" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>50</v>
+      <c r="A23" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>